<commit_message>
another f1 score fix
</commit_message>
<xml_diff>
--- a/VideoResultsNick.xlsx
+++ b/VideoResultsNick.xlsx
@@ -5,18 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nick_1/Desktop/University/1 - UWO Masters (2024 - ongoing)/Screen-Sight Paper/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nick_1/Dev/UWO/Screen-Sight/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34008A0D-BDBD-8C4B-A0F1-71F6C3C3CC36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB9FAD21-134A-A244-B8B6-4333AC84CEC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="2" xr2:uid="{08FD64ED-E66D-AB40-8BA8-4D60C0E42210}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20000" activeTab="2" xr2:uid="{08FD64ED-E66D-AB40-8BA8-4D60C0E42210}"/>
   </bookViews>
   <sheets>
     <sheet name="RawData" sheetId="1" r:id="rId1"/>
     <sheet name="Accuracy" sheetId="5" r:id="rId2"/>
-    <sheet name="F1Score" sheetId="6" r:id="rId3"/>
-    <sheet name="YoloImprovement " sheetId="4" r:id="rId4"/>
+    <sheet name="YoloImprovement " sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="27">
   <si>
     <t>Avg DPS</t>
   </si>
@@ -120,27 +119,6 @@
   </si>
   <si>
     <t>Accuracy calculated as (DETECTIONS/FRAMES)</t>
-  </si>
-  <si>
-    <t>YOLO F1 Score</t>
-  </si>
-  <si>
-    <t>ArUco F1 Score</t>
-  </si>
-  <si>
-    <t>F1 Score = TP / (TP + 0.5(FP + FN))</t>
-  </si>
-  <si>
-    <t>TP = detections</t>
-  </si>
-  <si>
-    <t>TN = impossible, phone is always present</t>
-  </si>
-  <si>
-    <t>FN = frames - detections</t>
-  </si>
-  <si>
-    <t>FP = detections - frames if detections &gt; frames</t>
   </si>
 </sst>
 </file>
@@ -588,6 +566,33 @@
     </xf>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
@@ -615,15 +620,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -634,24 +630,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1015,44 +993,44 @@
     <row r="1" spans="1:12" ht="31" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="17"/>
       <c r="B1" s="17"/>
-      <c r="C1" s="50" t="s">
+      <c r="C1" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="51"/>
-      <c r="E1" s="51"/>
-      <c r="F1" s="51"/>
-      <c r="G1" s="52"/>
-      <c r="H1" s="53" t="s">
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="40" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="54"/>
-      <c r="J1" s="54"/>
-      <c r="K1" s="54"/>
-      <c r="L1" s="55"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="41"/>
+      <c r="K1" s="41"/>
+      <c r="L1" s="42"/>
     </row>
     <row r="2" spans="1:12" ht="17" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="43" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="48"/>
-      <c r="C2" s="43" t="s">
+      <c r="B2" s="54"/>
+      <c r="C2" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="43" t="s">
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="44"/>
-      <c r="J2" s="44"/>
-      <c r="K2" s="44"/>
-      <c r="L2" s="45"/>
+      <c r="I2" s="38"/>
+      <c r="J2" s="38"/>
+      <c r="K2" s="38"/>
+      <c r="L2" s="39"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A3" s="35"/>
-      <c r="B3" s="49"/>
+      <c r="A3" s="44"/>
+      <c r="B3" s="55"/>
       <c r="C3" s="6" t="s">
         <v>1</v>
       </c>
@@ -1085,7 +1063,7 @@
       </c>
     </row>
     <row r="4" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A4" s="35"/>
+      <c r="A4" s="44"/>
       <c r="B4" s="4" t="s">
         <v>14</v>
       </c>
@@ -1121,7 +1099,7 @@
       </c>
     </row>
     <row r="5" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A5" s="35"/>
+      <c r="A5" s="44"/>
       <c r="B5" s="9" t="s">
         <v>13</v>
       </c>
@@ -1157,7 +1135,7 @@
       </c>
     </row>
     <row r="6" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A6" s="35"/>
+      <c r="A6" s="44"/>
       <c r="B6" s="4" t="s">
         <v>12</v>
       </c>
@@ -1193,7 +1171,7 @@
       </c>
     </row>
     <row r="7" spans="1:12" ht="18" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="35"/>
+      <c r="A7" s="44"/>
       <c r="B7" s="10" t="s">
         <v>11</v>
       </c>
@@ -1229,26 +1207,26 @@
       </c>
     </row>
     <row r="8" spans="1:12" ht="17" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="35"/>
-      <c r="B8" s="41"/>
-      <c r="C8" s="43" t="s">
+      <c r="A8" s="44"/>
+      <c r="B8" s="50"/>
+      <c r="C8" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="44"/>
-      <c r="E8" s="44"/>
-      <c r="F8" s="44"/>
-      <c r="G8" s="45"/>
-      <c r="H8" s="43" t="s">
+      <c r="D8" s="38"/>
+      <c r="E8" s="38"/>
+      <c r="F8" s="38"/>
+      <c r="G8" s="39"/>
+      <c r="H8" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="I8" s="44"/>
-      <c r="J8" s="44"/>
-      <c r="K8" s="44"/>
-      <c r="L8" s="45"/>
+      <c r="I8" s="38"/>
+      <c r="J8" s="38"/>
+      <c r="K8" s="38"/>
+      <c r="L8" s="39"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A9" s="35"/>
-      <c r="B9" s="42"/>
+      <c r="A9" s="44"/>
+      <c r="B9" s="51"/>
       <c r="C9" s="6" t="s">
         <v>1</v>
       </c>
@@ -1281,7 +1259,7 @@
       </c>
     </row>
     <row r="10" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A10" s="35"/>
+      <c r="A10" s="44"/>
       <c r="B10" s="5" t="s">
         <v>14</v>
       </c>
@@ -1317,7 +1295,7 @@
       </c>
     </row>
     <row r="11" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A11" s="35"/>
+      <c r="A11" s="44"/>
       <c r="B11" s="18" t="s">
         <v>13</v>
       </c>
@@ -1353,7 +1331,7 @@
       </c>
     </row>
     <row r="12" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A12" s="35"/>
+      <c r="A12" s="44"/>
       <c r="B12" s="5" t="s">
         <v>12</v>
       </c>
@@ -1389,7 +1367,7 @@
       </c>
     </row>
     <row r="13" spans="1:12" ht="18" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="36"/>
+      <c r="A13" s="45"/>
       <c r="B13" s="19" t="s">
         <v>11</v>
       </c>
@@ -1425,28 +1403,28 @@
       </c>
     </row>
     <row r="14" spans="1:12" ht="17" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="37" t="s">
+      <c r="A14" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="B14" s="46"/>
-      <c r="C14" s="43" t="s">
+      <c r="B14" s="52"/>
+      <c r="C14" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="D14" s="44"/>
-      <c r="E14" s="44"/>
-      <c r="F14" s="44"/>
-      <c r="G14" s="45"/>
-      <c r="H14" s="43" t="s">
+      <c r="D14" s="38"/>
+      <c r="E14" s="38"/>
+      <c r="F14" s="38"/>
+      <c r="G14" s="39"/>
+      <c r="H14" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="I14" s="44"/>
-      <c r="J14" s="44"/>
-      <c r="K14" s="44"/>
-      <c r="L14" s="45"/>
+      <c r="I14" s="38"/>
+      <c r="J14" s="38"/>
+      <c r="K14" s="38"/>
+      <c r="L14" s="39"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A15" s="38"/>
-      <c r="B15" s="47"/>
+      <c r="A15" s="47"/>
+      <c r="B15" s="53"/>
       <c r="C15" s="6" t="s">
         <v>1</v>
       </c>
@@ -1479,7 +1457,7 @@
       </c>
     </row>
     <row r="16" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A16" s="38"/>
+      <c r="A16" s="47"/>
       <c r="B16" s="4" t="s">
         <v>14</v>
       </c>
@@ -1515,7 +1493,7 @@
       </c>
     </row>
     <row r="17" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A17" s="38"/>
+      <c r="A17" s="47"/>
       <c r="B17" s="9" t="s">
         <v>13</v>
       </c>
@@ -1551,7 +1529,7 @@
       </c>
     </row>
     <row r="18" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A18" s="38"/>
+      <c r="A18" s="47"/>
       <c r="B18" s="4" t="s">
         <v>12</v>
       </c>
@@ -1587,7 +1565,7 @@
       </c>
     </row>
     <row r="19" spans="1:12" ht="18" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="38"/>
+      <c r="A19" s="47"/>
       <c r="B19" s="10" t="s">
         <v>11</v>
       </c>
@@ -1623,26 +1601,26 @@
       </c>
     </row>
     <row r="20" spans="1:12" ht="17" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="38"/>
-      <c r="B20" s="41"/>
-      <c r="C20" s="43" t="s">
+      <c r="A20" s="47"/>
+      <c r="B20" s="50"/>
+      <c r="C20" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="D20" s="44"/>
-      <c r="E20" s="44"/>
-      <c r="F20" s="44"/>
-      <c r="G20" s="45"/>
-      <c r="H20" s="43" t="s">
+      <c r="D20" s="38"/>
+      <c r="E20" s="38"/>
+      <c r="F20" s="38"/>
+      <c r="G20" s="39"/>
+      <c r="H20" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="I20" s="44"/>
-      <c r="J20" s="44"/>
-      <c r="K20" s="44"/>
-      <c r="L20" s="45"/>
+      <c r="I20" s="38"/>
+      <c r="J20" s="38"/>
+      <c r="K20" s="38"/>
+      <c r="L20" s="39"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A21" s="38"/>
-      <c r="B21" s="42"/>
+      <c r="A21" s="47"/>
+      <c r="B21" s="51"/>
       <c r="C21" s="6" t="s">
         <v>1</v>
       </c>
@@ -1675,7 +1653,7 @@
       </c>
     </row>
     <row r="22" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A22" s="38"/>
+      <c r="A22" s="47"/>
       <c r="B22" s="5" t="s">
         <v>14</v>
       </c>
@@ -1711,7 +1689,7 @@
       </c>
     </row>
     <row r="23" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A23" s="38"/>
+      <c r="A23" s="47"/>
       <c r="B23" s="18" t="s">
         <v>13</v>
       </c>
@@ -1747,7 +1725,7 @@
       </c>
     </row>
     <row r="24" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A24" s="38"/>
+      <c r="A24" s="47"/>
       <c r="B24" s="5" t="s">
         <v>12</v>
       </c>
@@ -1783,7 +1761,7 @@
       </c>
     </row>
     <row r="25" spans="1:12" ht="18" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="39"/>
+      <c r="A25" s="48"/>
       <c r="B25" s="19" t="s">
         <v>11</v>
       </c>
@@ -1820,75 +1798,69 @@
     </row>
     <row r="26" spans="1:12" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
     <row r="28" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B28" s="40" t="s">
+      <c r="B28" s="49" t="s">
         <v>15</v>
       </c>
-      <c r="C28" s="40"/>
-      <c r="D28" s="40"/>
-      <c r="E28" s="40"/>
-      <c r="F28" s="40"/>
-      <c r="G28" s="40"/>
-      <c r="H28" s="40"/>
-      <c r="I28" s="40"/>
-      <c r="J28" s="40"/>
-      <c r="K28" s="40"/>
+      <c r="C28" s="49"/>
+      <c r="D28" s="49"/>
+      <c r="E28" s="49"/>
+      <c r="F28" s="49"/>
+      <c r="G28" s="49"/>
+      <c r="H28" s="49"/>
+      <c r="I28" s="49"/>
+      <c r="J28" s="49"/>
+      <c r="K28" s="49"/>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="B29" s="40"/>
-      <c r="C29" s="40"/>
-      <c r="D29" s="40"/>
-      <c r="E29" s="40"/>
-      <c r="F29" s="40"/>
-      <c r="G29" s="40"/>
-      <c r="H29" s="40"/>
-      <c r="I29" s="40"/>
-      <c r="J29" s="40"/>
-      <c r="K29" s="40"/>
+      <c r="B29" s="49"/>
+      <c r="C29" s="49"/>
+      <c r="D29" s="49"/>
+      <c r="E29" s="49"/>
+      <c r="F29" s="49"/>
+      <c r="G29" s="49"/>
+      <c r="H29" s="49"/>
+      <c r="I29" s="49"/>
+      <c r="J29" s="49"/>
+      <c r="K29" s="49"/>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="B30" s="40"/>
-      <c r="C30" s="40"/>
-      <c r="D30" s="40"/>
-      <c r="E30" s="40"/>
-      <c r="F30" s="40"/>
-      <c r="G30" s="40"/>
-      <c r="H30" s="40"/>
-      <c r="I30" s="40"/>
-      <c r="J30" s="40"/>
-      <c r="K30" s="40"/>
+      <c r="B30" s="49"/>
+      <c r="C30" s="49"/>
+      <c r="D30" s="49"/>
+      <c r="E30" s="49"/>
+      <c r="F30" s="49"/>
+      <c r="G30" s="49"/>
+      <c r="H30" s="49"/>
+      <c r="I30" s="49"/>
+      <c r="J30" s="49"/>
+      <c r="K30" s="49"/>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="B31" s="40"/>
-      <c r="C31" s="40"/>
-      <c r="D31" s="40"/>
-      <c r="E31" s="40"/>
-      <c r="F31" s="40"/>
-      <c r="G31" s="40"/>
-      <c r="H31" s="40"/>
-      <c r="I31" s="40"/>
-      <c r="J31" s="40"/>
-      <c r="K31" s="40"/>
+      <c r="B31" s="49"/>
+      <c r="C31" s="49"/>
+      <c r="D31" s="49"/>
+      <c r="E31" s="49"/>
+      <c r="F31" s="49"/>
+      <c r="G31" s="49"/>
+      <c r="H31" s="49"/>
+      <c r="I31" s="49"/>
+      <c r="J31" s="49"/>
+      <c r="K31" s="49"/>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="B32" s="40"/>
-      <c r="C32" s="40"/>
-      <c r="D32" s="40"/>
-      <c r="E32" s="40"/>
-      <c r="F32" s="40"/>
-      <c r="G32" s="40"/>
-      <c r="H32" s="40"/>
-      <c r="I32" s="40"/>
-      <c r="J32" s="40"/>
-      <c r="K32" s="40"/>
+      <c r="B32" s="49"/>
+      <c r="C32" s="49"/>
+      <c r="D32" s="49"/>
+      <c r="E32" s="49"/>
+      <c r="F32" s="49"/>
+      <c r="G32" s="49"/>
+      <c r="H32" s="49"/>
+      <c r="I32" s="49"/>
+      <c r="J32" s="49"/>
+      <c r="K32" s="49"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="C1:G1"/>
-    <mergeCell ref="H8:L8"/>
-    <mergeCell ref="H2:L2"/>
-    <mergeCell ref="H1:L1"/>
-    <mergeCell ref="C2:G2"/>
-    <mergeCell ref="C8:G8"/>
     <mergeCell ref="A2:A13"/>
     <mergeCell ref="A14:A25"/>
     <mergeCell ref="B28:K32"/>
@@ -1900,6 +1872,12 @@
     <mergeCell ref="H14:L14"/>
     <mergeCell ref="B8:B9"/>
     <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C1:G1"/>
+    <mergeCell ref="H8:L8"/>
+    <mergeCell ref="H2:L2"/>
+    <mergeCell ref="H1:L1"/>
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="C8:G8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2202,313 +2180,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE59BAF5-37C2-144A-B695-3AE1F259F493}">
-  <dimension ref="A1:G22"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="2" max="5" width="16.6640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="57" t="s">
-        <v>27</v>
-      </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
-    </row>
-    <row r="2" spans="1:7" ht="68" x14ac:dyDescent="0.2">
-      <c r="A2" s="31" t="s">
-        <v>23</v>
-      </c>
-      <c r="B2" s="31" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2" s="31" t="s">
-        <v>17</v>
-      </c>
-      <c r="D2" s="31" t="s">
-        <v>18</v>
-      </c>
-      <c r="E2" s="31" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" s="32">
-        <v>0.25</v>
-      </c>
-      <c r="B3" s="27">
-        <f>RawData!F4/(RawData!F4 + (0.5 * (RawData!E4 - RawData!F4)))</f>
-        <v>0.99944165270798435</v>
-      </c>
-      <c r="C3" s="27">
-        <f>RawData!K4/(RawData!K4 + (0.5 * (RawData!J4 - RawData!K4)))</f>
-        <v>0.96079578700994739</v>
-      </c>
-      <c r="D3" s="27">
-        <f>RawData!F10/(RawData!F10 + (0.5 * (RawData!E10 - RawData!F10)))</f>
-        <v>0.96785930867192238</v>
-      </c>
-      <c r="E3" s="27">
-        <f>RawData!K10/(RawData!K10 + (0.5 * (RawData!J10 - RawData!K10)))</f>
-        <v>0.94384858044164033</v>
-      </c>
-      <c r="G3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="33">
-        <v>0.5</v>
-      </c>
-      <c r="B4" s="28">
-        <f>RawData!F5/(RawData!F5 + (0.5 * (RawData!E5 - RawData!F5)))</f>
-        <v>0.99944165270798435</v>
-      </c>
-      <c r="C4" s="28">
-        <f>RawData!K5/(RawData!K5 + (0.5 * (RawData!J5 - RawData!K5)))</f>
-        <v>0.99601593625498008</v>
-      </c>
-      <c r="D4" s="28">
-        <f>RawData!F11/(RawData!F11 + (0.5 * (RawData!E11 - RawData!F11)))</f>
-        <v>1.0016977928692699</v>
-      </c>
-      <c r="E4" s="28">
-        <f>RawData!K11/(RawData!K11 + (0.5 * (RawData!J11 - RawData!K11)))</f>
-        <v>0.87770700636942678</v>
-      </c>
-      <c r="G4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" s="32">
-        <v>0.75</v>
-      </c>
-      <c r="B5" s="27">
-        <f>RawData!F6/(RawData!F6 + (0.5 * (RawData!E6 - RawData!F6)))</f>
-        <v>1</v>
-      </c>
-      <c r="C5" s="27">
-        <f>RawData!K6/(RawData!K6 + (0.5 * (RawData!J6 - RawData!K6)))</f>
-        <v>0.98474178403755863</v>
-      </c>
-      <c r="D5" s="27">
-        <f>RawData!F12/(RawData!F12 + (0.5 * (RawData!E12 - RawData!F12)))</f>
-        <v>1.0045558086560364</v>
-      </c>
-      <c r="E5" s="27">
-        <f>RawData!K12/(RawData!K12 + (0.5 * (RawData!J12 - RawData!K12)))</f>
-        <v>0.79632248939179628</v>
-      </c>
-      <c r="G5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" s="33">
-        <v>1</v>
-      </c>
-      <c r="B6" s="28">
-        <f>RawData!F7/(RawData!F7 + (0.5 * (RawData!E7 - RawData!F7)))</f>
-        <v>0.99136442141623493</v>
-      </c>
-      <c r="C6" s="28">
-        <f>RawData!K7/(RawData!K7 + (0.5 * (RawData!J7 - RawData!K7)))</f>
-        <v>0.98456260720411659</v>
-      </c>
-      <c r="D6" s="28">
-        <f>RawData!F13/(RawData!F13 + (0.5 * (RawData!E13 - RawData!F13)))</f>
-        <v>1.005720823798627</v>
-      </c>
-      <c r="E6" s="28">
-        <f>RawData!K13/(RawData!K13 + (0.5 * (RawData!J13 - RawData!K13)))</f>
-        <v>0.8</v>
-      </c>
-      <c r="G6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" s="58"/>
-      <c r="B7" s="58"/>
-      <c r="C7" s="58"/>
-      <c r="D7" s="58"/>
-      <c r="E7" s="58"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" s="58"/>
-      <c r="B8" s="58"/>
-      <c r="C8" s="58"/>
-      <c r="D8" s="58"/>
-      <c r="E8" s="58"/>
-    </row>
-    <row r="9" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="56" t="s">
-        <v>28</v>
-      </c>
-      <c r="B9" s="56"/>
-      <c r="C9" s="56"/>
-      <c r="D9" s="56"/>
-      <c r="E9" s="56"/>
-    </row>
-    <row r="10" spans="1:7" ht="68" x14ac:dyDescent="0.2">
-      <c r="A10" s="31" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" s="31" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" s="31" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" s="31" t="s">
-        <v>18</v>
-      </c>
-      <c r="E10" s="31" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" s="32">
-        <v>0.25</v>
-      </c>
-      <c r="B11" s="27">
-        <f>RawData!F16/(RawData!F16 + (0.5 * (RawData!E16 - RawData!F16)))</f>
-        <v>0.42392260334212839</v>
-      </c>
-      <c r="C11" s="27">
-        <f>RawData!K16/(RawData!K16 + (0.5 * (RawData!J16 - RawData!K16)))</f>
-        <v>0.72961373390557938</v>
-      </c>
-      <c r="D11" s="27">
-        <f>RawData!F22/(RawData!F22 + (0.5 * (RawData!E22 - RawData!F22)))</f>
-        <v>0.33137254901960783</v>
-      </c>
-      <c r="E11" s="27">
-        <f>RawData!K22/(RawData!K22 + (0.5 * (RawData!J22 - RawData!K22)))</f>
-        <v>0.53028972783143113</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" s="33">
-        <v>0.5</v>
-      </c>
-      <c r="B12" s="28">
-        <f>RawData!F17/(RawData!F17 + (0.5 * (RawData!E17 - RawData!F17)))</f>
-        <v>0.9718875502008032</v>
-      </c>
-      <c r="C12" s="28">
-        <f>RawData!K17/(RawData!K17 + (0.5 * (RawData!J17 - RawData!K17)))</f>
-        <v>0.94623655913978499</v>
-      </c>
-      <c r="D12" s="28">
-        <f>RawData!F23/(RawData!F23 + (0.5 * (RawData!E23 - RawData!F23)))</f>
-        <v>0.65446224256292906</v>
-      </c>
-      <c r="E12" s="28">
-        <f>RawData!K23/(RawData!K23 + (0.5 * (RawData!J23 - RawData!K23)))</f>
-        <v>0.6266562743569758</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13" s="32">
-        <v>0.75</v>
-      </c>
-      <c r="B13" s="27">
-        <f>RawData!F18/(RawData!F18 + (0.5 * (RawData!E18 - RawData!F18)))</f>
-        <v>0.99592786503781272</v>
-      </c>
-      <c r="C13" s="27">
-        <f>RawData!K18/(RawData!K18 + (0.5 * (RawData!J18 - RawData!K18)))</f>
-        <v>0.96592946802151824</v>
-      </c>
-      <c r="D13" s="27">
-        <f>RawData!F24/(RawData!F24 + (0.5 * (RawData!E24 - RawData!F24)))</f>
-        <v>0.61599366587490101</v>
-      </c>
-      <c r="E13" s="27">
-        <f>RawData!K24/(RawData!K24 + (0.5 * (RawData!J24 - RawData!K24)))</f>
-        <v>0.57929883138564275</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A14" s="33">
-        <v>1</v>
-      </c>
-      <c r="B14" s="28">
-        <f>RawData!F19/(RawData!F19 + (0.5 * (RawData!E19 - RawData!F19)))</f>
-        <v>0.99194476409666288</v>
-      </c>
-      <c r="C14" s="28">
-        <f>RawData!K19/(RawData!K19 + (0.5 * (RawData!J19 - RawData!K19)))</f>
-        <v>0.9268882175226586</v>
-      </c>
-      <c r="D14" s="28">
-        <f>RawData!F25/(RawData!F25 + (0.5 * (RawData!E25 - RawData!F25)))</f>
-        <v>0.65583913379737047</v>
-      </c>
-      <c r="E14" s="28">
-        <f>RawData!K25/(RawData!K25 + (0.5 * (RawData!J25 - RawData!K25)))</f>
-        <v>0.61651676206050698</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A15" s="58"/>
-      <c r="B15" s="58"/>
-      <c r="C15" s="58"/>
-      <c r="D15" s="58"/>
-      <c r="E15" s="58"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" s="58"/>
-      <c r="B16" s="58"/>
-      <c r="C16" s="58"/>
-      <c r="D16" s="58"/>
-      <c r="E16" s="58"/>
-    </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B18" s="59" t="s">
-        <v>29</v>
-      </c>
-      <c r="C18" s="59"/>
-      <c r="D18" s="59"/>
-    </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B19" s="59"/>
-      <c r="C19" s="59"/>
-      <c r="D19" s="59"/>
-    </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B20" s="59"/>
-      <c r="C20" s="59"/>
-      <c r="D20" s="59"/>
-    </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B21" s="59"/>
-      <c r="C21" s="59"/>
-      <c r="D21" s="59"/>
-    </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B22" s="59"/>
-      <c r="C22" s="59"/>
-      <c r="D22" s="59"/>
-    </row>
-  </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A7:E8"/>
-    <mergeCell ref="A9:E9"/>
-    <mergeCell ref="A15:E16"/>
-    <mergeCell ref="B18:D22"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66A3D1B7-CEBE-4745-A6B4-0006F59E57EC}">
   <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>